<commit_message>
ui: fine-tune interface details
</commit_message>
<xml_diff>
--- a/public/form/出貨明細_範本.xlsx
+++ b/public/form/出貨明細_範本.xlsx
@@ -96,14 +96,14 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="微軟正黑體"/>
       <family val="2"/>
       <charset val="136"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="微軟正黑體"/>
       <family val="2"/>
@@ -111,7 +111,7 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="0"/>
       <name val="微軟正黑體"/>
       <family val="2"/>
@@ -458,7 +458,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="19.7" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="28.35" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.375" style="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.125" style="2" customWidth="1"/>
@@ -470,7 +470,7 @@
     <col min="9" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="28.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -482,7 +482,7 @@
       <c r="F1" s="4"/>
       <c r="H1" s="6"/>
     </row>
-    <row r="2" spans="1:8" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="28.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -493,7 +493,7 @@
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
     </row>
-    <row r="3" spans="1:8" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="28.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -504,7 +504,7 @@
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
     </row>
-    <row r="4" spans="1:8" s="9" customFormat="1" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" s="9" customFormat="1" ht="28.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
fix(shipping): correct shipping order detail table format and layout
</commit_message>
<xml_diff>
--- a/public/form/出貨明細_範本.xlsx
+++ b/public/form/出貨明細_範本.xlsx
@@ -70,7 +70,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -87,14 +87,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="微軟正黑體"/>
-      <family val="2"/>
-      <charset val="136"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="微軟正黑體"/>
@@ -105,6 +97,21 @@
       <b/>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="微軟正黑體"/>
       <family val="2"/>
       <charset val="136"/>
@@ -138,45 +145,51 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -461,72 +474,86 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="19.7" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.125" style="8" customWidth="1"/>
+    <col min="1" max="1" width="20.125" style="4" customWidth="1"/>
     <col min="2" max="2" width="35.125" style="1" customWidth="1"/>
     <col min="3" max="3" width="7.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5" style="8" customWidth="1"/>
-    <col min="5" max="5" width="1.5" style="12" customWidth="1"/>
+    <col min="4" max="4" width="7.5" style="4" customWidth="1"/>
+    <col min="5" max="5" width="1.5" style="6" customWidth="1"/>
     <col min="6" max="6" width="20.125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="35.125" style="4" customWidth="1"/>
-    <col min="8" max="9" width="7.5" style="4" customWidth="1"/>
-    <col min="10" max="16384" width="9" style="4"/>
+    <col min="7" max="7" width="35.125" style="2" customWidth="1"/>
+    <col min="8" max="9" width="7.5" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="3"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="2" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="5"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="2" t="s">
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="7" t="s">
         <v>6</v>
       </c>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
     </row>
     <row r="3" spans="1:9" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="6"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="2" t="s">
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="7" t="s">
         <v>9</v>
       </c>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
     </row>
-    <row r="4" spans="1:9" s="8" customFormat="1" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:9" s="4" customFormat="1" ht="19.7" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="11"/>
-      <c r="F4" s="7" t="s">
+      <c r="E4" s="5"/>
+      <c r="F4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="3" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>